<commit_message>
notes and debug stuff
</commit_message>
<xml_diff>
--- a/Notes/datamapping-MOVES.xlsx
+++ b/Notes/datamapping-MOVES.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\cygwin64\home\scrawford\silvermirror-local\Notes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49512027-EB7B-4A91-BA1C-BBBEBE64B99F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{318E2B62-4B8F-42A0-984C-60D7B6DA38FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{1982F562-5184-46C6-89BD-68E4E108BC42}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4742" uniqueCount="1393">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4767" uniqueCount="1398">
   <si>
     <t>bug</t>
   </si>
@@ -3882,15 +3882,9 @@
     <t>HORN_ATTACK, poison</t>
   </si>
   <si>
-    <t>CHARM no heart</t>
-  </si>
-  <si>
     <t>THRASH, fighting</t>
   </si>
   <si>
-    <t>EGG_BOMB, grass</t>
-  </si>
-  <si>
     <t>FURY_ATTACK, ice, w/ crystal hits</t>
   </si>
   <si>
@@ -3903,12 +3897,6 @@
     <t>SAND_ATTACK but SPIKE_CANNON spikes (change?)</t>
   </si>
   <si>
-    <t>PSYBEAM, water</t>
-  </si>
-  <si>
-    <t>WATERFALL, water</t>
-  </si>
-  <si>
     <t>RAPID_SPIN (maybe metal intro)</t>
   </si>
   <si>
@@ -3924,9 +3912,6 @@
     <t>SUPERSONIC, SACRED_FIRE on target</t>
   </si>
   <si>
-    <t>SWEET_SCENT, all gfx are leaves, hit</t>
-  </si>
-  <si>
     <t>SLASH, dark</t>
   </si>
   <si>
@@ -3987,6 +3972,9 @@
     <t>statdown</t>
   </si>
   <si>
+    <t>color</t>
+  </si>
+  <si>
     <t>; aa</t>
   </si>
   <si>
@@ -4219,6 +4207,33 @@
   </si>
   <si>
     <t>EFFECT</t>
+  </si>
+  <si>
+    <t>user doesn't wobble?</t>
+  </si>
+  <si>
+    <t>PSYWAVE, water (psybeam)</t>
+  </si>
+  <si>
+    <t>no endure?</t>
+  </si>
+  <si>
+    <t>hits</t>
+  </si>
+  <si>
+    <t>BARRAGE, green</t>
+  </si>
+  <si>
+    <t>WATERFALL reversed</t>
+  </si>
+  <si>
+    <t>POWDER_SNOW, gfx_reflect, green</t>
+  </si>
+  <si>
+    <t>ACID, ground</t>
+  </si>
+  <si>
+    <t>hex</t>
   </si>
 </sst>
 </file>
@@ -4425,7 +4440,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -4544,6 +4559,7 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -6531,7 +6547,7 @@
         <v>1268</v>
       </c>
       <c r="J14" t="s">
-        <v>1310</v>
+        <v>1305</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
@@ -6571,7 +6587,7 @@
         <v>1268</v>
       </c>
       <c r="J16" t="s">
-        <v>1312</v>
+        <v>1307</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
@@ -6619,7 +6635,7 @@
         <v>1267</v>
       </c>
       <c r="J19" t="s">
-        <v>1313</v>
+        <v>1308</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
@@ -6648,7 +6664,7 @@
         <v>1268</v>
       </c>
       <c r="J20" t="s">
-        <v>1306</v>
+        <v>1301</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
@@ -6765,10 +6781,10 @@
         <v>1267</v>
       </c>
       <c r="I26" s="3" t="s">
-        <v>1314</v>
+        <v>1309</v>
       </c>
       <c r="J26" t="s">
-        <v>1281</v>
+        <v>1280</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
@@ -7167,7 +7183,7 @@
         <v>1268</v>
       </c>
       <c r="J50" t="s">
-        <v>1309</v>
+        <v>1304</v>
       </c>
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.25">
@@ -7239,11 +7255,11 @@
       <c r="H55" t="s">
         <v>1267</v>
       </c>
-      <c r="I55" s="4" t="s">
-        <v>1311</v>
+      <c r="I55" s="1" t="s">
+        <v>1268</v>
       </c>
       <c r="J55" t="s">
-        <v>1308</v>
+        <v>1303</v>
       </c>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.25">
@@ -7557,7 +7573,7 @@
         <v>1056</v>
       </c>
     </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A81" s="4" t="s">
         <v>841</v>
       </c>
@@ -7568,7 +7584,7 @@
         <v>977</v>
       </c>
     </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A82" s="4" t="s">
         <v>842</v>
       </c>
@@ -7579,7 +7595,7 @@
         <v>978</v>
       </c>
     </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A83" s="4" t="s">
         <v>843</v>
       </c>
@@ -7590,7 +7606,7 @@
         <v>979</v>
       </c>
     </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A84" s="4" t="s">
         <v>844</v>
       </c>
@@ -7601,7 +7617,7 @@
         <v>980</v>
       </c>
     </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A85" s="4" t="s">
         <v>845</v>
       </c>
@@ -7612,7 +7628,7 @@
         <v>981</v>
       </c>
     </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A86" s="4" t="s">
         <v>846</v>
       </c>
@@ -7623,7 +7639,7 @@
         <v>982</v>
       </c>
     </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A87" s="4" t="s">
         <v>847</v>
       </c>
@@ -7634,7 +7650,7 @@
         <v>983</v>
       </c>
     </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A88" s="4" t="s">
         <v>848</v>
       </c>
@@ -7645,7 +7661,7 @@
         <v>984</v>
       </c>
     </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A89" s="4" t="s">
         <v>849</v>
       </c>
@@ -7656,7 +7672,7 @@
         <v>985</v>
       </c>
     </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A90" s="4" t="s">
         <v>850</v>
       </c>
@@ -7667,7 +7683,7 @@
         <v>986</v>
       </c>
     </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A91" s="4" t="s">
         <v>851</v>
       </c>
@@ -7678,7 +7694,7 @@
         <v>1057</v>
       </c>
     </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A92" s="4" t="s">
         <v>852</v>
       </c>
@@ -7689,7 +7705,7 @@
         <v>1058</v>
       </c>
     </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A93" s="4" t="s">
         <v>853</v>
       </c>
@@ -7700,7 +7716,7 @@
         <v>1059</v>
       </c>
     </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A94" s="4" t="s">
         <v>854</v>
       </c>
@@ -7711,7 +7727,7 @@
         <v>1060</v>
       </c>
     </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A95" s="4" t="s">
         <v>855</v>
       </c>
@@ -7721,8 +7737,11 @@
       <c r="C95" t="s">
         <v>1061</v>
       </c>
-    </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="I95" s="4" t="s">
+        <v>1310</v>
+      </c>
+    </row>
+    <row r="96" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A96" s="4" t="s">
         <v>856</v>
       </c>
@@ -7755,8 +7774,8 @@
       <c r="H97" t="s">
         <v>1267</v>
       </c>
-      <c r="I97" s="4" t="s">
-        <v>1311</v>
+      <c r="I97" s="1" t="s">
+        <v>1268</v>
       </c>
       <c r="J97" t="s">
         <v>89</v>
@@ -7839,11 +7858,11 @@
       <c r="H103" t="s">
         <v>1267</v>
       </c>
-      <c r="I103" s="4" t="s">
-        <v>1311</v>
+      <c r="I103" s="1" t="s">
+        <v>1268</v>
       </c>
       <c r="J103" t="s">
-        <v>1389</v>
+        <v>1385</v>
       </c>
     </row>
     <row r="104" spans="1:10" x14ac:dyDescent="0.25">
@@ -7945,11 +7964,11 @@
       <c r="H111" t="s">
         <v>1267</v>
       </c>
-      <c r="I111" s="4" t="s">
-        <v>1311</v>
+      <c r="I111" s="1" t="s">
+        <v>1268</v>
       </c>
       <c r="J111" t="s">
-        <v>1280</v>
+        <v>1389</v>
       </c>
     </row>
     <row r="112" spans="1:10" x14ac:dyDescent="0.25">
@@ -8068,11 +8087,11 @@
       <c r="H120" t="s">
         <v>1267</v>
       </c>
-      <c r="I120" s="4" t="s">
-        <v>1311</v>
+      <c r="I120" s="1" t="s">
+        <v>1268</v>
       </c>
       <c r="J120" t="s">
-        <v>1388</v>
+        <v>1384</v>
       </c>
     </row>
     <row r="121" spans="1:10" x14ac:dyDescent="0.25">
@@ -8109,10 +8128,10 @@
         <v>1267</v>
       </c>
       <c r="I122" s="4" t="s">
-        <v>1311</v>
+        <v>1306</v>
       </c>
       <c r="J122" t="s">
-        <v>1282</v>
+        <v>1393</v>
       </c>
     </row>
     <row r="123" spans="1:10" x14ac:dyDescent="0.25">
@@ -8207,7 +8226,7 @@
         <v>1268</v>
       </c>
       <c r="J129" t="s">
-        <v>1307</v>
+        <v>1302</v>
       </c>
     </row>
     <row r="130" spans="1:10" x14ac:dyDescent="0.25">
@@ -8243,11 +8262,11 @@
       <c r="H131" t="s">
         <v>1267</v>
       </c>
-      <c r="I131" s="4" t="s">
-        <v>1311</v>
+      <c r="I131" s="1" t="s">
+        <v>1268</v>
       </c>
       <c r="J131" t="s">
-        <v>1387</v>
+        <v>1383</v>
       </c>
     </row>
     <row r="132" spans="1:10" x14ac:dyDescent="0.25">
@@ -8273,10 +8292,10 @@
         <v>1267</v>
       </c>
       <c r="I132" s="4" t="s">
-        <v>1311</v>
+        <v>1392</v>
       </c>
       <c r="J132" t="s">
-        <v>1283</v>
+        <v>1281</v>
       </c>
     </row>
     <row r="133" spans="1:10" x14ac:dyDescent="0.25">
@@ -8301,8 +8320,11 @@
       <c r="H133" t="s">
         <v>1267</v>
       </c>
-      <c r="I133" s="4" t="s">
-        <v>1311</v>
+      <c r="I133" s="1" t="s">
+        <v>1268</v>
+      </c>
+      <c r="J133" t="s">
+        <v>1391</v>
       </c>
     </row>
     <row r="134" spans="1:10" x14ac:dyDescent="0.25">
@@ -8315,8 +8337,8 @@
       <c r="C134" t="s">
         <v>1012</v>
       </c>
-      <c r="I134" s="4" t="s">
-        <v>1311</v>
+      <c r="I134" s="1" t="s">
+        <v>1268</v>
       </c>
     </row>
     <row r="135" spans="1:10" x14ac:dyDescent="0.25">
@@ -8345,7 +8367,7 @@
         <v>1268</v>
       </c>
       <c r="J135" t="s">
-        <v>1391</v>
+        <v>1387</v>
       </c>
     </row>
     <row r="136" spans="1:10" x14ac:dyDescent="0.25">
@@ -8381,11 +8403,11 @@
       <c r="H137" t="s">
         <v>1267</v>
       </c>
-      <c r="I137" s="4" t="s">
-        <v>1311</v>
+      <c r="I137" s="1" t="s">
+        <v>1268</v>
       </c>
       <c r="J137" t="s">
-        <v>1284</v>
+        <v>1282</v>
       </c>
     </row>
     <row r="138" spans="1:10" x14ac:dyDescent="0.25">
@@ -8432,8 +8454,8 @@
       <c r="H140" t="s">
         <v>1267</v>
       </c>
-      <c r="I140" s="4" t="s">
-        <v>1311</v>
+      <c r="I140" s="1" t="s">
+        <v>1268</v>
       </c>
       <c r="J140" t="s">
         <v>1279</v>
@@ -8465,7 +8487,7 @@
         <v>1268</v>
       </c>
       <c r="J141" t="s">
-        <v>1286</v>
+        <v>1284</v>
       </c>
     </row>
     <row r="142" spans="1:10" x14ac:dyDescent="0.25">
@@ -8490,7 +8512,7 @@
         <v>1239</v>
       </c>
       <c r="D143" s="3" t="s">
-        <v>1392</v>
+        <v>1388</v>
       </c>
       <c r="E143" t="s">
         <v>1263</v>
@@ -8508,7 +8530,7 @@
         <v>1268</v>
       </c>
       <c r="J143" t="s">
-        <v>1285</v>
+        <v>1283</v>
       </c>
     </row>
     <row r="144" spans="1:10" x14ac:dyDescent="0.25">
@@ -8521,9 +8543,12 @@
       <c r="C144" t="s">
         <v>1080</v>
       </c>
+      <c r="I144" s="1" t="s">
+        <v>1268</v>
+      </c>
     </row>
     <row r="145" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A145" t="s">
+      <c r="A145" s="4" t="s">
         <v>905</v>
       </c>
       <c r="B145" t="s">
@@ -8534,7 +8559,7 @@
       </c>
     </row>
     <row r="146" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A146" t="s">
+      <c r="A146" s="4" t="s">
         <v>906</v>
       </c>
       <c r="B146" s="3" t="s">
@@ -8555,12 +8580,15 @@
       <c r="H146" t="s">
         <v>1267</v>
       </c>
+      <c r="I146" s="4" t="s">
+        <v>1306</v>
+      </c>
       <c r="J146" t="s">
-        <v>1287</v>
+        <v>1390</v>
       </c>
     </row>
     <row r="147" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A147" t="s">
+      <c r="A147" s="4" t="s">
         <v>907</v>
       </c>
       <c r="B147" t="s">
@@ -8571,7 +8599,7 @@
       </c>
     </row>
     <row r="148" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A148" t="s">
+      <c r="A148" s="4" t="s">
         <v>908</v>
       </c>
       <c r="B148" t="s">
@@ -8582,7 +8610,7 @@
       </c>
     </row>
     <row r="149" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A149" t="s">
+      <c r="A149" s="4" t="s">
         <v>909</v>
       </c>
       <c r="B149" t="s">
@@ -8593,7 +8621,7 @@
       </c>
     </row>
     <row r="150" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A150" t="s">
+      <c r="A150" s="4" t="s">
         <v>910</v>
       </c>
       <c r="B150" s="3" t="s">
@@ -8614,12 +8642,15 @@
       <c r="H150" t="s">
         <v>1267</v>
       </c>
+      <c r="I150" s="4" t="s">
+        <v>1306</v>
+      </c>
       <c r="J150" t="s">
         <v>146</v>
       </c>
     </row>
     <row r="151" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A151" t="s">
+      <c r="A151" s="4" t="s">
         <v>911</v>
       </c>
       <c r="B151" t="s">
@@ -8630,7 +8661,7 @@
       </c>
     </row>
     <row r="152" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A152" t="s">
+      <c r="A152" s="4" t="s">
         <v>912</v>
       </c>
       <c r="B152" s="3" t="s">
@@ -8651,12 +8682,15 @@
       <c r="H152" t="s">
         <v>1267</v>
       </c>
+      <c r="I152" s="4" t="s">
+        <v>1306</v>
+      </c>
       <c r="J152" t="s">
-        <v>1288</v>
+        <v>1394</v>
       </c>
     </row>
     <row r="153" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A153" t="s">
+      <c r="A153" s="4" t="s">
         <v>913</v>
       </c>
       <c r="B153" t="s">
@@ -8667,7 +8701,7 @@
       </c>
     </row>
     <row r="154" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A154" t="s">
+      <c r="A154" s="4" t="s">
         <v>914</v>
       </c>
       <c r="B154" s="3" t="s">
@@ -8688,12 +8722,15 @@
       <c r="H154" t="s">
         <v>1267</v>
       </c>
+      <c r="I154" s="4" t="s">
+        <v>1306</v>
+      </c>
       <c r="J154" t="s">
-        <v>1304</v>
+        <v>1299</v>
       </c>
     </row>
     <row r="155" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A155" t="s">
+      <c r="A155" s="4" t="s">
         <v>915</v>
       </c>
       <c r="B155" s="3" t="s">
@@ -8714,12 +8751,15 @@
       <c r="H155" t="s">
         <v>1267</v>
       </c>
+      <c r="I155" s="1" t="s">
+        <v>1268</v>
+      </c>
       <c r="J155" t="s">
-        <v>1390</v>
+        <v>1386</v>
       </c>
     </row>
     <row r="156" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A156" t="s">
+      <c r="A156" s="4" t="s">
         <v>916</v>
       </c>
       <c r="B156" t="s">
@@ -8730,7 +8770,7 @@
       </c>
     </row>
     <row r="157" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A157" t="s">
+      <c r="A157" s="4" t="s">
         <v>917</v>
       </c>
       <c r="B157" t="s">
@@ -8741,7 +8781,7 @@
       </c>
     </row>
     <row r="158" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A158" t="s">
+      <c r="A158" s="4" t="s">
         <v>918</v>
       </c>
       <c r="B158" t="s">
@@ -8752,7 +8792,7 @@
       </c>
     </row>
     <row r="159" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A159" t="s">
+      <c r="A159" s="4" t="s">
         <v>919</v>
       </c>
       <c r="B159" t="s">
@@ -8763,7 +8803,7 @@
       </c>
     </row>
     <row r="160" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A160" t="s">
+      <c r="A160" s="4" t="s">
         <v>920</v>
       </c>
       <c r="B160" t="s">
@@ -8774,7 +8814,7 @@
       </c>
     </row>
     <row r="161" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A161" t="s">
+      <c r="A161" s="4" t="s">
         <v>921</v>
       </c>
       <c r="B161" t="s">
@@ -8785,7 +8825,7 @@
       </c>
     </row>
     <row r="162" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A162" t="s">
+      <c r="A162" s="4" t="s">
         <v>922</v>
       </c>
       <c r="B162" t="s">
@@ -8796,7 +8836,7 @@
       </c>
     </row>
     <row r="163" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A163" t="s">
+      <c r="A163" s="4" t="s">
         <v>923</v>
       </c>
       <c r="B163" t="s">
@@ -8807,7 +8847,7 @@
       </c>
     </row>
     <row r="164" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A164" t="s">
+      <c r="A164" s="4" t="s">
         <v>924</v>
       </c>
       <c r="B164" t="s">
@@ -8818,7 +8858,7 @@
       </c>
     </row>
     <row r="165" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A165" t="s">
+      <c r="A165" s="4" t="s">
         <v>925</v>
       </c>
       <c r="B165" t="s">
@@ -8829,7 +8869,7 @@
       </c>
     </row>
     <row r="166" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A166" t="s">
+      <c r="A166" s="4" t="s">
         <v>926</v>
       </c>
       <c r="B166" s="3" t="s">
@@ -8850,12 +8890,15 @@
       <c r="H166" t="s">
         <v>1267</v>
       </c>
+      <c r="I166" s="4" t="s">
+        <v>1306</v>
+      </c>
       <c r="J166" t="s">
-        <v>1289</v>
+        <v>1285</v>
       </c>
     </row>
     <row r="167" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A167" t="s">
+      <c r="A167" s="4" t="s">
         <v>1194</v>
       </c>
       <c r="B167" t="s">
@@ -8866,7 +8909,7 @@
       </c>
     </row>
     <row r="168" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A168" t="s">
+      <c r="A168" s="4" t="s">
         <v>1195</v>
       </c>
       <c r="B168" s="3" t="s">
@@ -8887,12 +8930,15 @@
       <c r="H168" t="s">
         <v>1267</v>
       </c>
+      <c r="I168" s="4" t="s">
+        <v>1306</v>
+      </c>
       <c r="J168" t="s">
-        <v>1290</v>
+        <v>1286</v>
       </c>
     </row>
     <row r="169" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A169" t="s">
+      <c r="A169" s="4" t="s">
         <v>1196</v>
       </c>
       <c r="B169" t="s">
@@ -8903,7 +8949,7 @@
       </c>
     </row>
     <row r="170" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A170" t="s">
+      <c r="A170" s="4" t="s">
         <v>1197</v>
       </c>
       <c r="B170" s="3" t="s">
@@ -8927,13 +8973,16 @@
       <c r="H170" t="s">
         <v>1267</v>
       </c>
+      <c r="I170" s="4" t="s">
+        <v>1306</v>
+      </c>
       <c r="J170" t="s">
-        <v>1291</v>
+        <v>1287</v>
       </c>
     </row>
     <row r="171" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A171" t="s">
-        <v>1315</v>
+      <c r="A171" s="4" t="s">
+        <v>1311</v>
       </c>
       <c r="B171" s="3" t="s">
         <v>1106</v>
@@ -8953,13 +9002,16 @@
       <c r="H171" t="s">
         <v>1267</v>
       </c>
+      <c r="I171" s="4" t="s">
+        <v>1306</v>
+      </c>
       <c r="J171" t="s">
-        <v>1292</v>
+        <v>1288</v>
       </c>
     </row>
     <row r="172" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A172" t="s">
-        <v>1316</v>
+      <c r="A172" s="4" t="s">
+        <v>1312</v>
       </c>
       <c r="B172" t="s">
         <v>1107</v>
@@ -8969,8 +9021,8 @@
       </c>
     </row>
     <row r="173" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A173" t="s">
-        <v>1317</v>
+      <c r="A173" s="4" t="s">
+        <v>1313</v>
       </c>
       <c r="B173" t="s">
         <v>1108</v>
@@ -8980,8 +9032,8 @@
       </c>
     </row>
     <row r="174" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A174" t="s">
-        <v>1318</v>
+      <c r="A174" s="4" t="s">
+        <v>1314</v>
       </c>
       <c r="B174" t="s">
         <v>1109</v>
@@ -8991,8 +9043,8 @@
       </c>
     </row>
     <row r="175" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A175" t="s">
-        <v>1319</v>
+      <c r="A175" s="4" t="s">
+        <v>1315</v>
       </c>
       <c r="B175" t="s">
         <v>1110</v>
@@ -9002,8 +9054,8 @@
       </c>
     </row>
     <row r="176" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A176" t="s">
-        <v>1320</v>
+      <c r="A176" s="4" t="s">
+        <v>1316</v>
       </c>
       <c r="B176" t="s">
         <v>1111</v>
@@ -9013,7 +9065,7 @@
       </c>
     </row>
     <row r="177" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A177" t="s">
+      <c r="A177" s="4" t="s">
         <v>1198</v>
       </c>
       <c r="B177" s="3" t="s">
@@ -9034,12 +9086,15 @@
       <c r="H177" t="s">
         <v>1267</v>
       </c>
+      <c r="I177" s="4" t="s">
+        <v>1306</v>
+      </c>
       <c r="J177" t="s">
-        <v>1293</v>
+        <v>1289</v>
       </c>
     </row>
     <row r="178" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A178" t="s">
+      <c r="A178" s="4" t="s">
         <v>1199</v>
       </c>
       <c r="B178" t="s">
@@ -9050,7 +9105,7 @@
       </c>
     </row>
     <row r="179" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A179" t="s">
+      <c r="A179" s="4" t="s">
         <v>1200</v>
       </c>
       <c r="B179" s="3" t="s">
@@ -9071,12 +9126,15 @@
       <c r="H179" t="s">
         <v>1267</v>
       </c>
+      <c r="I179" s="1" t="s">
+        <v>1268</v>
+      </c>
       <c r="J179" t="s">
-        <v>1294</v>
+        <v>1395</v>
       </c>
     </row>
     <row r="180" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A180" t="s">
+      <c r="A180" s="4" t="s">
         <v>1201</v>
       </c>
       <c r="B180" s="3" t="s">
@@ -9101,14 +9159,14 @@
         <v>1267</v>
       </c>
       <c r="I180" s="4" t="s">
-        <v>1311</v>
+        <v>1306</v>
       </c>
       <c r="J180" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="181" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A181" t="s">
+      <c r="A181" s="4" t="s">
         <v>1202</v>
       </c>
       <c r="B181" s="3" t="s">
@@ -9132,12 +9190,15 @@
       <c r="H181" t="s">
         <v>1267</v>
       </c>
+      <c r="I181" s="58" t="s">
+        <v>1268</v>
+      </c>
       <c r="J181" t="s">
-        <v>1295</v>
+        <v>1290</v>
       </c>
     </row>
     <row r="182" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A182" t="s">
+      <c r="A182" s="4" t="s">
         <v>1203</v>
       </c>
       <c r="B182" t="s">
@@ -9148,7 +9209,7 @@
       </c>
     </row>
     <row r="183" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A183" t="s">
+      <c r="A183" s="4" t="s">
         <v>1204</v>
       </c>
       <c r="B183" t="s">
@@ -9159,7 +9220,7 @@
       </c>
     </row>
     <row r="184" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A184" t="s">
+      <c r="A184" s="4" t="s">
         <v>1205</v>
       </c>
       <c r="B184" t="s">
@@ -9170,7 +9231,7 @@
       </c>
     </row>
     <row r="185" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A185" t="s">
+      <c r="A185" s="4" t="s">
         <v>1206</v>
       </c>
       <c r="B185" t="s">
@@ -9181,7 +9242,7 @@
       </c>
     </row>
     <row r="186" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A186" t="s">
+      <c r="A186" s="4" t="s">
         <v>1207</v>
       </c>
       <c r="B186" t="s">
@@ -9192,7 +9253,7 @@
       </c>
     </row>
     <row r="187" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A187" t="s">
+      <c r="A187" s="4" t="s">
         <v>1208</v>
       </c>
       <c r="B187" s="3" t="s">
@@ -9213,12 +9274,15 @@
       <c r="H187" t="s">
         <v>1267</v>
       </c>
+      <c r="I187" s="58" t="s">
+        <v>1268</v>
+      </c>
       <c r="J187" t="s">
-        <v>1296</v>
+        <v>1291</v>
       </c>
     </row>
     <row r="188" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A188" t="s">
+      <c r="A188" s="4" t="s">
         <v>1209</v>
       </c>
       <c r="B188" t="s">
@@ -9229,7 +9293,7 @@
       </c>
     </row>
     <row r="189" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A189" t="s">
+      <c r="A189" s="4" t="s">
         <v>1210</v>
       </c>
       <c r="B189" t="s">
@@ -9240,7 +9304,7 @@
       </c>
     </row>
     <row r="190" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A190" t="s">
+      <c r="A190" s="4" t="s">
         <v>1211</v>
       </c>
       <c r="B190" t="s">
@@ -9251,8 +9315,8 @@
       </c>
     </row>
     <row r="191" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A191" t="s">
-        <v>1321</v>
+      <c r="A191" s="4" t="s">
+        <v>1317</v>
       </c>
       <c r="B191" t="s">
         <v>1126</v>
@@ -9262,8 +9326,8 @@
       </c>
     </row>
     <row r="192" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A192" t="s">
-        <v>1322</v>
+      <c r="A192" s="4" t="s">
+        <v>1318</v>
       </c>
       <c r="B192" t="s">
         <v>1127</v>
@@ -9273,8 +9337,8 @@
       </c>
     </row>
     <row r="193" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A193" t="s">
-        <v>1323</v>
+      <c r="A193" s="4" t="s">
+        <v>1319</v>
       </c>
       <c r="B193" t="s">
         <v>1128</v>
@@ -9284,8 +9348,8 @@
       </c>
     </row>
     <row r="194" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A194" t="s">
-        <v>1325</v>
+      <c r="A194" s="4" t="s">
+        <v>1321</v>
       </c>
       <c r="B194" t="s">
         <v>1129</v>
@@ -9295,8 +9359,8 @@
       </c>
     </row>
     <row r="195" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A195" t="s">
-        <v>1326</v>
+      <c r="A195" s="4" t="s">
+        <v>1322</v>
       </c>
       <c r="B195" t="s">
         <v>1130</v>
@@ -9306,8 +9370,8 @@
       </c>
     </row>
     <row r="196" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A196" t="s">
-        <v>1327</v>
+      <c r="A196" s="4" t="s">
+        <v>1323</v>
       </c>
       <c r="B196" t="s">
         <v>1131</v>
@@ -9317,8 +9381,8 @@
       </c>
     </row>
     <row r="197" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A197" t="s">
-        <v>1328</v>
+      <c r="A197" s="4" t="s">
+        <v>1324</v>
       </c>
       <c r="B197" t="s">
         <v>1132</v>
@@ -9328,8 +9392,8 @@
       </c>
     </row>
     <row r="198" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A198" t="s">
-        <v>1329</v>
+      <c r="A198" s="4" t="s">
+        <v>1325</v>
       </c>
       <c r="B198" s="3" t="s">
         <v>1133</v>
@@ -9349,13 +9413,16 @@
       <c r="H198" t="s">
         <v>1267</v>
       </c>
+      <c r="I198" s="58" t="s">
+        <v>1268</v>
+      </c>
       <c r="J198" t="s">
-        <v>1297</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="199" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A199" t="s">
-        <v>1330</v>
+      <c r="A199" s="4" t="s">
+        <v>1326</v>
       </c>
       <c r="B199" s="3" t="s">
         <v>1134</v>
@@ -9375,10 +9442,13 @@
       <c r="H199" t="s">
         <v>1267</v>
       </c>
+      <c r="I199" s="58" t="s">
+        <v>1268</v>
+      </c>
     </row>
     <row r="200" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A200" t="s">
-        <v>1331</v>
+      <c r="A200" s="4" t="s">
+        <v>1327</v>
       </c>
       <c r="B200" t="s">
         <v>1135</v>
@@ -9388,8 +9458,8 @@
       </c>
     </row>
     <row r="201" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A201" t="s">
-        <v>1332</v>
+      <c r="A201" s="4" t="s">
+        <v>1328</v>
       </c>
       <c r="B201" t="s">
         <v>1136</v>
@@ -9399,8 +9469,8 @@
       </c>
     </row>
     <row r="202" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A202" t="s">
-        <v>1333</v>
+      <c r="A202" s="4" t="s">
+        <v>1329</v>
       </c>
       <c r="B202" t="s">
         <v>1137</v>
@@ -9410,8 +9480,8 @@
       </c>
     </row>
     <row r="203" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A203" t="s">
-        <v>1334</v>
+      <c r="A203" s="4" t="s">
+        <v>1330</v>
       </c>
       <c r="B203" t="s">
         <v>1138</v>
@@ -9421,8 +9491,8 @@
       </c>
     </row>
     <row r="204" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A204" t="s">
-        <v>1335</v>
+      <c r="A204" s="4" t="s">
+        <v>1331</v>
       </c>
       <c r="B204" t="s">
         <v>1139</v>
@@ -9432,8 +9502,8 @@
       </c>
     </row>
     <row r="205" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A205" t="s">
-        <v>1386</v>
+      <c r="A205" s="4" t="s">
+        <v>1382</v>
       </c>
       <c r="B205" t="s">
         <v>1140</v>
@@ -9443,8 +9513,8 @@
       </c>
     </row>
     <row r="206" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A206" t="s">
-        <v>1336</v>
+      <c r="A206" s="4" t="s">
+        <v>1332</v>
       </c>
       <c r="B206" t="s">
         <v>1141</v>
@@ -9454,8 +9524,8 @@
       </c>
     </row>
     <row r="207" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A207" t="s">
-        <v>1337</v>
+      <c r="A207" s="4" t="s">
+        <v>1333</v>
       </c>
       <c r="B207" t="s">
         <v>1142</v>
@@ -9465,8 +9535,8 @@
       </c>
     </row>
     <row r="208" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A208" t="s">
-        <v>1324</v>
+      <c r="A208" s="4" t="s">
+        <v>1320</v>
       </c>
       <c r="B208" t="s">
         <v>1143</v>
@@ -9476,8 +9546,8 @@
       </c>
     </row>
     <row r="209" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A209" t="s">
-        <v>1338</v>
+      <c r="A209" s="4" t="s">
+        <v>1334</v>
       </c>
       <c r="B209" s="3" t="s">
         <v>1144</v>
@@ -9497,10 +9567,16 @@
       <c r="H209" t="s">
         <v>1267</v>
       </c>
+      <c r="I209" s="4" t="s">
+        <v>1306</v>
+      </c>
+      <c r="J209" t="s">
+        <v>1396</v>
+      </c>
     </row>
     <row r="210" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A210" t="s">
-        <v>1339</v>
+      <c r="A210" s="4" t="s">
+        <v>1335</v>
       </c>
       <c r="B210" t="s">
         <v>1145</v>
@@ -9510,8 +9586,8 @@
       </c>
     </row>
     <row r="211" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A211" t="s">
-        <v>1340</v>
+      <c r="A211" s="4" t="s">
+        <v>1336</v>
       </c>
       <c r="B211" t="s">
         <v>1146</v>
@@ -9521,8 +9597,8 @@
       </c>
     </row>
     <row r="212" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A212" t="s">
-        <v>1341</v>
+      <c r="A212" s="4" t="s">
+        <v>1337</v>
       </c>
       <c r="B212" t="s">
         <v>1147</v>
@@ -9532,8 +9608,8 @@
       </c>
     </row>
     <row r="213" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A213" t="s">
-        <v>1342</v>
+      <c r="A213" s="4" t="s">
+        <v>1338</v>
       </c>
       <c r="B213" t="s">
         <v>1148</v>
@@ -9543,8 +9619,8 @@
       </c>
     </row>
     <row r="214" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A214" t="s">
-        <v>1343</v>
+      <c r="A214" s="4" t="s">
+        <v>1339</v>
       </c>
       <c r="B214" t="s">
         <v>1149</v>
@@ -9554,8 +9630,8 @@
       </c>
     </row>
     <row r="215" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A215" t="s">
-        <v>1344</v>
+      <c r="A215" s="4" t="s">
+        <v>1340</v>
       </c>
       <c r="B215" t="s">
         <v>1150</v>
@@ -9565,8 +9641,8 @@
       </c>
     </row>
     <row r="216" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A216" t="s">
-        <v>1345</v>
+      <c r="A216" s="4" t="s">
+        <v>1341</v>
       </c>
       <c r="B216" t="s">
         <v>1151</v>
@@ -9576,8 +9652,8 @@
       </c>
     </row>
     <row r="217" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A217" t="s">
-        <v>1346</v>
+      <c r="A217" s="4" t="s">
+        <v>1342</v>
       </c>
       <c r="B217" s="3" t="s">
         <v>1152</v>
@@ -9597,13 +9673,16 @@
       <c r="H217" t="s">
         <v>1267</v>
       </c>
+      <c r="I217" s="58" t="s">
+        <v>1268</v>
+      </c>
       <c r="J217" t="s">
-        <v>1298</v>
+        <v>1293</v>
       </c>
     </row>
     <row r="218" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A218" t="s">
-        <v>1347</v>
+      <c r="A218" s="4" t="s">
+        <v>1343</v>
       </c>
       <c r="B218" s="3" t="s">
         <v>1153</v>
@@ -9623,13 +9702,16 @@
       <c r="H218" t="s">
         <v>1267</v>
       </c>
+      <c r="I218" s="58" t="s">
+        <v>1268</v>
+      </c>
       <c r="J218" t="s">
-        <v>1299</v>
+        <v>1294</v>
       </c>
     </row>
     <row r="219" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A219" t="s">
-        <v>1348</v>
+      <c r="A219" s="4" t="s">
+        <v>1344</v>
       </c>
       <c r="B219" s="3" t="s">
         <v>1154</v>
@@ -9649,13 +9731,16 @@
       <c r="H219" t="s">
         <v>1267</v>
       </c>
+      <c r="I219" s="4" t="s">
+        <v>1397</v>
+      </c>
       <c r="J219" t="s">
-        <v>533</v>
+        <v>327</v>
       </c>
     </row>
     <row r="220" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A220" t="s">
-        <v>1349</v>
+      <c r="A220" s="4" t="s">
+        <v>1345</v>
       </c>
       <c r="B220" t="s">
         <v>1155</v>
@@ -9665,8 +9750,8 @@
       </c>
     </row>
     <row r="221" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A221" t="s">
-        <v>1350</v>
+      <c r="A221" s="4" t="s">
+        <v>1346</v>
       </c>
       <c r="B221" t="s">
         <v>1156</v>
@@ -9676,8 +9761,8 @@
       </c>
     </row>
     <row r="222" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A222" t="s">
-        <v>1385</v>
+      <c r="A222" s="4" t="s">
+        <v>1381</v>
       </c>
       <c r="B222" t="s">
         <v>1157</v>
@@ -9687,8 +9772,8 @@
       </c>
     </row>
     <row r="223" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A223" t="s">
-        <v>1351</v>
+      <c r="A223" s="4" t="s">
+        <v>1347</v>
       </c>
       <c r="B223" t="s">
         <v>1158</v>
@@ -9698,8 +9783,8 @@
       </c>
     </row>
     <row r="224" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A224" t="s">
-        <v>1352</v>
+      <c r="A224" s="4" t="s">
+        <v>1348</v>
       </c>
       <c r="B224" t="s">
         <v>1159</v>
@@ -9709,8 +9794,8 @@
       </c>
     </row>
     <row r="225" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A225" t="s">
-        <v>1353</v>
+      <c r="A225" s="4" t="s">
+        <v>1349</v>
       </c>
       <c r="B225" t="s">
         <v>1160</v>
@@ -9720,8 +9805,8 @@
       </c>
     </row>
     <row r="226" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A226" t="s">
-        <v>1354</v>
+      <c r="A226" s="4" t="s">
+        <v>1350</v>
       </c>
       <c r="B226" t="s">
         <v>1161</v>
@@ -9731,8 +9816,8 @@
       </c>
     </row>
     <row r="227" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A227" t="s">
-        <v>1355</v>
+      <c r="A227" s="4" t="s">
+        <v>1351</v>
       </c>
       <c r="B227" t="s">
         <v>1162</v>
@@ -9742,8 +9827,8 @@
       </c>
     </row>
     <row r="228" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A228" t="s">
-        <v>1356</v>
+      <c r="A228" s="4" t="s">
+        <v>1352</v>
       </c>
       <c r="B228" t="s">
         <v>1163</v>
@@ -9753,8 +9838,8 @@
       </c>
     </row>
     <row r="229" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A229" t="s">
-        <v>1357</v>
+      <c r="A229" s="4" t="s">
+        <v>1353</v>
       </c>
       <c r="B229" t="s">
         <v>1164</v>
@@ -9764,8 +9849,8 @@
       </c>
     </row>
     <row r="230" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A230" t="s">
-        <v>1358</v>
+      <c r="A230" s="4" t="s">
+        <v>1354</v>
       </c>
       <c r="B230" t="s">
         <v>1165</v>
@@ -9775,8 +9860,8 @@
       </c>
     </row>
     <row r="231" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A231" t="s">
-        <v>1359</v>
+      <c r="A231" s="4" t="s">
+        <v>1355</v>
       </c>
       <c r="B231" t="s">
         <v>1166</v>
@@ -9786,8 +9871,8 @@
       </c>
     </row>
     <row r="232" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A232" t="s">
-        <v>1360</v>
+      <c r="A232" s="4" t="s">
+        <v>1356</v>
       </c>
       <c r="B232" t="s">
         <v>1167</v>
@@ -9797,8 +9882,8 @@
       </c>
     </row>
     <row r="233" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A233" t="s">
-        <v>1361</v>
+      <c r="A233" s="4" t="s">
+        <v>1357</v>
       </c>
       <c r="B233" t="s">
         <v>1168</v>
@@ -9808,8 +9893,8 @@
       </c>
     </row>
     <row r="234" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A234" t="s">
-        <v>1362</v>
+      <c r="A234" s="4" t="s">
+        <v>1358</v>
       </c>
       <c r="B234" s="3" t="s">
         <v>1169</v>
@@ -9829,13 +9914,16 @@
       <c r="H234" t="s">
         <v>1267</v>
       </c>
+      <c r="I234" s="4" t="s">
+        <v>1306</v>
+      </c>
       <c r="J234" t="s">
-        <v>1305</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="235" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A235" t="s">
-        <v>1363</v>
+      <c r="A235" s="4" t="s">
+        <v>1359</v>
       </c>
       <c r="B235" t="s">
         <v>1170</v>
@@ -9845,8 +9933,8 @@
       </c>
     </row>
     <row r="236" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A236" t="s">
-        <v>1364</v>
+      <c r="A236" s="4" t="s">
+        <v>1360</v>
       </c>
       <c r="B236" t="s">
         <v>1171</v>
@@ -9856,8 +9944,8 @@
       </c>
     </row>
     <row r="237" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A237" t="s">
-        <v>1365</v>
+      <c r="A237" s="4" t="s">
+        <v>1361</v>
       </c>
       <c r="B237" t="s">
         <v>1172</v>
@@ -9867,8 +9955,8 @@
       </c>
     </row>
     <row r="238" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A238" t="s">
-        <v>1366</v>
+      <c r="A238" s="4" t="s">
+        <v>1362</v>
       </c>
       <c r="B238" t="s">
         <v>1173</v>
@@ -9878,8 +9966,8 @@
       </c>
     </row>
     <row r="239" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A239" t="s">
-        <v>1384</v>
+      <c r="A239" s="4" t="s">
+        <v>1380</v>
       </c>
       <c r="B239" t="s">
         <v>1174</v>
@@ -9889,8 +9977,8 @@
       </c>
     </row>
     <row r="240" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A240" t="s">
-        <v>1367</v>
+      <c r="A240" s="4" t="s">
+        <v>1363</v>
       </c>
       <c r="B240" t="s">
         <v>1175</v>
@@ -9900,8 +9988,8 @@
       </c>
     </row>
     <row r="241" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A241" t="s">
-        <v>1368</v>
+      <c r="A241" s="4" t="s">
+        <v>1364</v>
       </c>
       <c r="B241" t="s">
         <v>1176</v>
@@ -9911,8 +9999,8 @@
       </c>
     </row>
     <row r="242" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A242" t="s">
-        <v>1369</v>
+      <c r="A242" s="4" t="s">
+        <v>1365</v>
       </c>
       <c r="B242" t="s">
         <v>1177</v>
@@ -9922,8 +10010,8 @@
       </c>
     </row>
     <row r="243" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A243" t="s">
-        <v>1370</v>
+      <c r="A243" s="4" t="s">
+        <v>1366</v>
       </c>
       <c r="B243" t="s">
         <v>1178</v>
@@ -9933,8 +10021,8 @@
       </c>
     </row>
     <row r="244" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A244" t="s">
-        <v>1371</v>
+      <c r="A244" s="4" t="s">
+        <v>1367</v>
       </c>
       <c r="B244" t="s">
         <v>1179</v>
@@ -9944,8 +10032,8 @@
       </c>
     </row>
     <row r="245" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A245" t="s">
-        <v>1372</v>
+      <c r="A245" s="4" t="s">
+        <v>1368</v>
       </c>
       <c r="B245" s="3" t="s">
         <v>1193</v>
@@ -9966,15 +10054,15 @@
         <v>1267</v>
       </c>
       <c r="I245" s="4" t="s">
-        <v>1311</v>
+        <v>1306</v>
       </c>
       <c r="J245" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="246" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A246" t="s">
-        <v>1373</v>
+      <c r="A246" s="4" t="s">
+        <v>1369</v>
       </c>
       <c r="B246" t="s">
         <v>1181</v>
@@ -9984,8 +10072,8 @@
       </c>
     </row>
     <row r="247" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A247" t="s">
-        <v>1374</v>
+      <c r="A247" s="4" t="s">
+        <v>1370</v>
       </c>
       <c r="B247" t="s">
         <v>1182</v>
@@ -9995,8 +10083,8 @@
       </c>
     </row>
     <row r="248" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A248" t="s">
-        <v>1375</v>
+      <c r="A248" s="4" t="s">
+        <v>1371</v>
       </c>
       <c r="B248" t="s">
         <v>1183</v>
@@ -10006,8 +10094,8 @@
       </c>
     </row>
     <row r="249" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A249" t="s">
-        <v>1376</v>
+      <c r="A249" s="4" t="s">
+        <v>1372</v>
       </c>
       <c r="B249" t="s">
         <v>1184</v>
@@ -10017,8 +10105,8 @@
       </c>
     </row>
     <row r="250" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A250" t="s">
-        <v>1377</v>
+      <c r="A250" s="4" t="s">
+        <v>1373</v>
       </c>
       <c r="B250" s="55" t="s">
         <v>1185</v>
@@ -10033,8 +10121,8 @@
       </c>
     </row>
     <row r="251" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A251" t="s">
-        <v>1378</v>
+      <c r="A251" s="4" t="s">
+        <v>1374</v>
       </c>
       <c r="B251" t="s">
         <v>1186</v>
@@ -10044,8 +10132,8 @@
       </c>
     </row>
     <row r="252" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A252" t="s">
-        <v>1379</v>
+      <c r="A252" s="4" t="s">
+        <v>1375</v>
       </c>
       <c r="B252" s="3" t="s">
         <v>1187</v>
@@ -10065,13 +10153,16 @@
       <c r="H252" t="s">
         <v>1267</v>
       </c>
+      <c r="I252" s="4" t="s">
+        <v>1306</v>
+      </c>
       <c r="J252" t="s">
-        <v>1300</v>
+        <v>1295</v>
       </c>
     </row>
     <row r="253" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A253" t="s">
-        <v>1380</v>
+        <v>1376</v>
       </c>
       <c r="C253" s="54" t="s">
         <v>1189</v>
@@ -10089,12 +10180,12 @@
         <v>1267</v>
       </c>
       <c r="J253" t="s">
-        <v>1302</v>
+        <v>1297</v>
       </c>
     </row>
     <row r="254" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A254" t="s">
-        <v>1381</v>
+        <v>1377</v>
       </c>
       <c r="C254" s="54" t="s">
         <v>1190</v>
@@ -10112,12 +10203,12 @@
         <v>1267</v>
       </c>
       <c r="J254" t="s">
-        <v>1301</v>
+        <v>1296</v>
       </c>
     </row>
     <row r="255" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A255" t="s">
-        <v>1382</v>
+        <v>1378</v>
       </c>
       <c r="C255" s="54" t="s">
         <v>1188</v>
@@ -10135,12 +10226,12 @@
         <v>1267</v>
       </c>
       <c r="J255" t="s">
-        <v>1303</v>
+        <v>1298</v>
       </c>
     </row>
     <row r="256" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A256" t="s">
-        <v>1383</v>
+        <v>1379</v>
       </c>
       <c r="C256" t="s">
         <v>1092</v>
@@ -23901,8 +23992,8 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="C8:C14">
-    <cfRule type="duplicateValues" dxfId="137" priority="88"/>
-    <cfRule type="duplicateValues" dxfId="136" priority="89"/>
+    <cfRule type="duplicateValues" dxfId="137" priority="89"/>
+    <cfRule type="duplicateValues" dxfId="136" priority="88"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C15:C18">
     <cfRule type="duplicateValues" dxfId="135" priority="92"/>
@@ -23921,8 +24012,8 @@
     <cfRule type="duplicateValues" dxfId="130" priority="84"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C43:C47">
-    <cfRule type="duplicateValues" dxfId="129" priority="82"/>
-    <cfRule type="duplicateValues" dxfId="128" priority="83"/>
+    <cfRule type="duplicateValues" dxfId="129" priority="83"/>
+    <cfRule type="duplicateValues" dxfId="128" priority="82"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C48:C53">
     <cfRule type="duplicateValues" dxfId="127" priority="80"/>
@@ -23934,8 +24025,8 @@
     <cfRule type="duplicateValues" dxfId="125" priority="79"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C59:C62">
-    <cfRule type="duplicateValues" dxfId="124" priority="77"/>
-    <cfRule type="duplicateValues" dxfId="123" priority="78"/>
+    <cfRule type="duplicateValues" dxfId="124" priority="78"/>
+    <cfRule type="duplicateValues" dxfId="123" priority="77"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C63:C70">
     <cfRule type="duplicateValues" dxfId="122" priority="94"/>
@@ -23974,8 +24065,8 @@
     <cfRule type="duplicateValues" dxfId="111" priority="519"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="L18:L21">
-    <cfRule type="duplicateValues" dxfId="110" priority="110"/>
-    <cfRule type="duplicateValues" dxfId="109" priority="111"/>
+    <cfRule type="duplicateValues" dxfId="110" priority="111"/>
+    <cfRule type="duplicateValues" dxfId="109" priority="110"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="L23:L30">
     <cfRule type="duplicateValues" dxfId="108" priority="515"/>
@@ -23987,8 +24078,8 @@
     <cfRule type="duplicateValues" dxfId="106" priority="507"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="L44:L48">
-    <cfRule type="duplicateValues" dxfId="105" priority="106"/>
-    <cfRule type="duplicateValues" dxfId="104" priority="107"/>
+    <cfRule type="duplicateValues" dxfId="105" priority="107"/>
+    <cfRule type="duplicateValues" dxfId="104" priority="106"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="L50:L51">
     <cfRule type="duplicateValues" dxfId="103" priority="105"/>
@@ -24082,12 +24173,12 @@
     <cfRule type="duplicateValues" dxfId="73" priority="66"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="U13">
-    <cfRule type="duplicateValues" dxfId="72" priority="64"/>
-    <cfRule type="duplicateValues" dxfId="71" priority="65"/>
+    <cfRule type="duplicateValues" dxfId="72" priority="65"/>
+    <cfRule type="duplicateValues" dxfId="71" priority="64"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="U14:U15">
-    <cfRule type="duplicateValues" dxfId="70" priority="62"/>
-    <cfRule type="duplicateValues" dxfId="69" priority="63"/>
+    <cfRule type="duplicateValues" dxfId="70" priority="63"/>
+    <cfRule type="duplicateValues" dxfId="69" priority="62"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="U16">
     <cfRule type="duplicateValues" dxfId="68" priority="61"/>
@@ -24111,16 +24202,16 @@
     <cfRule type="duplicateValues" dxfId="62" priority="55"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="U29">
-    <cfRule type="duplicateValues" dxfId="61" priority="53"/>
-    <cfRule type="duplicateValues" dxfId="60" priority="54"/>
+    <cfRule type="duplicateValues" dxfId="61" priority="54"/>
+    <cfRule type="duplicateValues" dxfId="60" priority="53"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="U30">
-    <cfRule type="duplicateValues" dxfId="59" priority="51"/>
-    <cfRule type="duplicateValues" dxfId="58" priority="52"/>
+    <cfRule type="duplicateValues" dxfId="59" priority="52"/>
+    <cfRule type="duplicateValues" dxfId="58" priority="51"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="U31">
-    <cfRule type="duplicateValues" dxfId="57" priority="49"/>
-    <cfRule type="duplicateValues" dxfId="56" priority="50"/>
+    <cfRule type="duplicateValues" dxfId="57" priority="50"/>
+    <cfRule type="duplicateValues" dxfId="56" priority="49"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="U33">
     <cfRule type="duplicateValues" dxfId="55" priority="47"/>
@@ -24143,8 +24234,8 @@
     <cfRule type="duplicateValues" dxfId="48" priority="42"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="U43:U45">
-    <cfRule type="duplicateValues" dxfId="47" priority="40"/>
-    <cfRule type="duplicateValues" dxfId="46" priority="41"/>
+    <cfRule type="duplicateValues" dxfId="47" priority="41"/>
+    <cfRule type="duplicateValues" dxfId="46" priority="40"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="U47">
     <cfRule type="duplicateValues" dxfId="45" priority="39"/>

</xml_diff>